<commit_message>
Criação da planilha para a implementação do diario de bordo
</commit_message>
<xml_diff>
--- a/Diario_De_Bordo.xlsx
+++ b/Diario_De_Bordo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CAMARGO\Music\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F69ED6BB-5B67-4E6E-8957-9AEBB8AC86CE}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F54F5DA-D8D0-446B-BE5F-D96D0F616E9B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" xr2:uid="{2188939B-C38A-46B0-BBE4-B78761095C61}"/>
   </bookViews>
@@ -26,9 +26,6 @@
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="12">
-  <si>
-    <t>TUIUTI</t>
-  </si>
   <si>
     <t>OK</t>
   </si>
@@ -61,6 +58,9 @@
   </si>
   <si>
     <t>Criação de uma tabela de planejamento.</t>
+  </si>
+  <si>
+    <t>TRABALHO DS</t>
   </si>
 </sst>
 </file>
@@ -786,7 +786,7 @@
   <sheetData>
     <row r="8" spans="6:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="F8" s="13" t="s">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="G8" s="14"/>
       <c r="H8" s="14"/>
@@ -799,28 +799,28 @@
     </row>
     <row r="9" spans="6:14" x14ac:dyDescent="0.25">
       <c r="F9" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="G9" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="G9" s="5" t="s">
+      <c r="H9" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="I9" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="H9" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="I9" s="5" t="s">
+      <c r="J9" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="J9" s="5" t="s">
+      <c r="K9" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="K9" s="5" t="s">
+      <c r="L9" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="L9" s="5" t="s">
+      <c r="M9" s="5" t="s">
         <v>8</v>
-      </c>
-      <c r="M9" s="5" t="s">
-        <v>9</v>
       </c>
       <c r="N9" s="2"/>
     </row>
@@ -829,10 +829,10 @@
         <v>1</v>
       </c>
       <c r="G10" s="19" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="H10" s="19" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I10" s="20">
         <v>46107</v>
@@ -841,13 +841,13 @@
         <v>46108</v>
       </c>
       <c r="K10" s="21" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L10" s="20">
         <v>46108</v>
       </c>
       <c r="M10" s="21" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N10" s="3"/>
     </row>

</xml_diff>